<commit_message>
Perfis de reporte e ajuste de armazens
</commit_message>
<xml_diff>
--- a/server/ALIAS.xlsx
+++ b/server/ALIAS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felip\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\felip\Documents\GitHub\Catalogo-de-itens\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CDC129B-BBA6-4CD5-BC8D-29F6D68AAC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{865650FC-51DE-460E-811B-046103A52F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-132" windowWidth="23256" windowHeight="12456" xr2:uid="{A0FD097D-02CF-4DC1-A130-9A4BAAEDE9E5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A0FD097D-02CF-4DC1-A130-9A4BAAEDE9E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>WH - APE.S APEADOS PALMELA</t>
   </si>
@@ -174,6 +174,75 @@
   </si>
   <si>
     <t>DESCRIÇÃO FICHEIRO</t>
+  </si>
+  <si>
+    <t>OUTROS</t>
+  </si>
+  <si>
+    <t>LISBOA</t>
+  </si>
+  <si>
+    <t>PORTO</t>
+  </si>
+  <si>
+    <t>LEIRIA</t>
+  </si>
+  <si>
+    <t>FARO</t>
+  </si>
+  <si>
+    <t>GUARDA</t>
+  </si>
+  <si>
+    <t>MADEIRA</t>
+  </si>
+  <si>
+    <t>PONTA DELGADA</t>
+  </si>
+  <si>
+    <t>MONTALVO</t>
+  </si>
+  <si>
+    <t>ST.MARIA DA FEIRA</t>
+  </si>
+  <si>
+    <t>BRAGA</t>
+  </si>
+  <si>
+    <t>PALMELA</t>
+  </si>
+  <si>
+    <t>APEADOS LISBOA</t>
+  </si>
+  <si>
+    <t>APEADOS PORTO</t>
+  </si>
+  <si>
+    <t>APEADOS LEIRIA</t>
+  </si>
+  <si>
+    <t>APEADOS FARO</t>
+  </si>
+  <si>
+    <t>APEADOS GUARDA</t>
+  </si>
+  <si>
+    <t>APEADOS MADEIRA</t>
+  </si>
+  <si>
+    <t>APEADOS MONTALVO</t>
+  </si>
+  <si>
+    <t>APEADOS BRAGA</t>
+  </si>
+  <si>
+    <t>APEADOS PALMELA</t>
+  </si>
+  <si>
+    <t>APEADOS ST.MARIA</t>
+  </si>
+  <si>
+    <t>APEADOS P. DELGADA</t>
   </si>
 </sst>
 </file>
@@ -573,195 +642,264 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AFC5138-349C-45A3-87D1-AA91725C005C}">
-  <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultColWidth="87" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr defaultColWidth="87" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="39.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>0</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>